<commit_message>
SPM-94: Refresh the traceability matrix for the test run
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-94_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-94_Test_Cases.xlsx
@@ -1526,11 +1526,7 @@
       <c r="A17" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>a6fb199</t>
-        </is>
-      </c>
+      <c r="B17" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1670,11 +1666,7 @@
       <c r="A17" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>a6fb199</t>
-        </is>
-      </c>
+      <c r="B17" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1814,11 +1806,7 @@
       <c r="A17" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>a6fb199</t>
-        </is>
-      </c>
+      <c r="B17" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1958,11 +1946,7 @@
       <c r="A17" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>a6fb199</t>
-        </is>
-      </c>
+      <c r="B17" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2102,11 +2086,7 @@
       <c r="A17" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>a6fb199</t>
-        </is>
-      </c>
+      <c r="B17" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2246,11 +2226,7 @@
       <c r="A17" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>a6fb199</t>
-        </is>
-      </c>
+      <c r="B17" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2390,11 +2366,7 @@
       <c r="A17" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>a6fb199</t>
-        </is>
-      </c>
+      <c r="B17" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2534,11 +2506,7 @@
       <c r="A17" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>a6fb199</t>
-        </is>
-      </c>
+      <c r="B17" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2678,11 +2646,7 @@
       <c r="A17" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>a6fb199</t>
-        </is>
-      </c>
+      <c r="B17" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2822,11 +2786,7 @@
       <c r="A17" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>a6fb199</t>
-        </is>
-      </c>
+      <c r="B17" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
SPM-94: Record the second manual test run (10 pass)
Also restores the Commit cells of the first run's blocks (a6fb199), which
8e96570 blanked when Excel re-saved the workbook over the hook's edit.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-94_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-94_Test_Cases.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\IS212\docs\test-cases\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\krist\Documents\GitHub\IS212\docs\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CC944A3-285E-4BCE-A2C9-6AF47A78BDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77421384-D10B-4FDA-83EE-AF7E14D25F2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" firstSheet="8" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14730" yWindow="-16200" windowWidth="14610" windowHeight="15585" firstSheet="5" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="122">
   <si>
     <t>Story</t>
   </si>
@@ -553,6 +553,12 @@
   <si>
     <t>Kayalvizhi</t>
   </si>
+  <si>
+    <t>a6fb199</t>
+  </si>
+  <si>
+    <t>Kristen</t>
+  </si>
 </sst>
 </file>
 
@@ -561,7 +567,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -596,6 +602,20 @@
       <color rgb="FF1155CC"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -622,7 +642,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -684,11 +704,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -714,13 +747,19 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -938,7 +977,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I23"/>
-  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -951,11 +990,11 @@
     <col min="9" max="9" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="B1" s="13" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="14"/>
@@ -966,7 +1005,7 @@
       <c r="H1" s="14"/>
       <c r="I1" s="15"/>
     </row>
-    <row r="3" spans="1:9" ht="13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>2</v>
       </c>
@@ -995,7 +1034,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="25" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>11</v>
       </c>
@@ -1020,7 +1059,7 @@
       <c r="H4" s="9"/>
       <c r="I4" s="9"/>
     </row>
-    <row r="5" spans="1:9" ht="25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>18</v>
       </c>
@@ -1045,7 +1084,7 @@
       <c r="H5" s="9"/>
       <c r="I5" s="9"/>
     </row>
-    <row r="6" spans="1:9" ht="25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>21</v>
       </c>
@@ -1070,7 +1109,7 @@
       <c r="H6" s="9"/>
       <c r="I6" s="9"/>
     </row>
-    <row r="7" spans="1:9" ht="25" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
         <v>24</v>
       </c>
@@ -1095,7 +1134,7 @@
       <c r="H7" s="9"/>
       <c r="I7" s="9"/>
     </row>
-    <row r="8" spans="1:9" ht="25" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>29</v>
       </c>
@@ -1120,7 +1159,7 @@
       <c r="H8" s="9"/>
       <c r="I8" s="9"/>
     </row>
-    <row r="9" spans="1:9" ht="25" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>33</v>
       </c>
@@ -1145,7 +1184,7 @@
       <c r="H9" s="9"/>
       <c r="I9" s="9"/>
     </row>
-    <row r="10" spans="1:9" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>37</v>
       </c>
@@ -1170,7 +1209,7 @@
       <c r="H10" s="9"/>
       <c r="I10" s="9"/>
     </row>
-    <row r="11" spans="1:9" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>40</v>
       </c>
@@ -1195,7 +1234,7 @@
       <c r="H11" s="9"/>
       <c r="I11" s="9"/>
     </row>
-    <row r="12" spans="1:9" ht="25" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
         <v>43</v>
       </c>
@@ -1220,7 +1259,7 @@
       <c r="H12" s="9"/>
       <c r="I12" s="9"/>
     </row>
-    <row r="13" spans="1:9" ht="25" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
         <v>47</v>
       </c>
@@ -1245,136 +1284,136 @@
       <c r="H13" s="9"/>
       <c r="I13" s="9"/>
     </row>
-    <row r="16" spans="1:9" ht="13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B16" s="16" t="s">
+      <c r="B16" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C16" s="14"/>
       <c r="D16" s="15"/>
-      <c r="E16" s="16" t="s">
+      <c r="E16" s="13" t="s">
         <v>54</v>
       </c>
       <c r="F16" s="15"/>
     </row>
-    <row r="17" spans="1:6" ht="71.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" ht="71.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="B17" s="16" t="s">
         <v>55</v>
       </c>
       <c r="C17" s="14"/>
       <c r="D17" s="15"/>
-      <c r="E17" s="13" t="s">
+      <c r="E17" s="16" t="s">
         <v>56</v>
       </c>
       <c r="F17" s="15"/>
     </row>
-    <row r="18" spans="1:6" ht="71.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" ht="71.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="16" t="s">
         <v>57</v>
       </c>
       <c r="C18" s="14"/>
       <c r="D18" s="15"/>
-      <c r="E18" s="13" t="s">
+      <c r="E18" s="16" t="s">
         <v>58</v>
       </c>
       <c r="F18" s="15"/>
     </row>
-    <row r="19" spans="1:6" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="B19" s="13" t="s">
+      <c r="B19" s="16" t="s">
         <v>60</v>
       </c>
       <c r="C19" s="14"/>
       <c r="D19" s="15"/>
-      <c r="E19" s="13" t="s">
+      <c r="E19" s="16" t="s">
         <v>25</v>
       </c>
       <c r="F19" s="15"/>
     </row>
-    <row r="20" spans="1:6" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="B20" s="13" t="s">
+      <c r="B20" s="16" t="s">
         <v>62</v>
       </c>
       <c r="C20" s="14"/>
       <c r="D20" s="15"/>
-      <c r="E20" s="13" t="s">
+      <c r="E20" s="16" t="s">
         <v>30</v>
       </c>
       <c r="F20" s="15"/>
     </row>
-    <row r="21" spans="1:6" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="B21" s="13" t="s">
+      <c r="B21" s="16" t="s">
         <v>64</v>
       </c>
       <c r="C21" s="14"/>
       <c r="D21" s="15"/>
-      <c r="E21" s="13" t="s">
+      <c r="E21" s="16" t="s">
         <v>65</v>
       </c>
       <c r="F21" s="15"/>
     </row>
-    <row r="22" spans="1:6" ht="71.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" ht="71.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="B22" s="16" t="s">
         <v>67</v>
       </c>
       <c r="C22" s="14"/>
       <c r="D22" s="15"/>
-      <c r="E22" s="13" t="s">
+      <c r="E22" s="16" t="s">
         <v>68</v>
       </c>
       <c r="F22" s="15"/>
     </row>
-    <row r="23" spans="1:6" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="B23" s="13" t="s">
+      <c r="B23" s="16" t="s">
         <v>70</v>
       </c>
       <c r="C23" s="14"/>
       <c r="D23" s="15"/>
-      <c r="E23" s="13" t="s">
+      <c r="E23" s="16" t="s">
         <v>44</v>
       </c>
       <c r="F23" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="B21:D21"/>
     <mergeCell ref="B1:I1"/>
     <mergeCell ref="B16:D16"/>
     <mergeCell ref="B20:D20"/>
     <mergeCell ref="B19:D19"/>
     <mergeCell ref="E20:F20"/>
     <mergeCell ref="E16:F16"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="E19:F19"/>
     <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="B21:D21"/>
     <mergeCell ref="E17:F17"/>
   </mergeCells>
   <hyperlinks>
@@ -1398,20 +1437,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>71</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -1419,7 +1458,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>72</v>
       </c>
@@ -1427,7 +1466,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>73</v>
       </c>
@@ -1435,7 +1474,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="152.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="152.55000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>75</v>
       </c>
@@ -1443,7 +1482,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>77</v>
       </c>
@@ -1451,7 +1490,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="179.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="179.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>79</v>
       </c>
@@ -1459,7 +1498,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>81</v>
       </c>
@@ -1467,7 +1506,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>83</v>
       </c>
@@ -1475,14 +1514,14 @@
         <v>46318</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>71</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="162.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="171.6" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>84</v>
       </c>
@@ -1490,7 +1529,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>85</v>
       </c>
@@ -1498,7 +1537,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>86</v>
       </c>
@@ -1506,7 +1545,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>87</v>
       </c>
@@ -1514,7 +1553,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>88</v>
       </c>
@@ -1522,11 +1561,69 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="3"/>
+      <c r="B17" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="171.6" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B21" s="18" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B22" s="19" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B23" s="19" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B24" s="20">
+        <v>46321</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B25" s="19" t="inlineStr">
+        <is>
+          <t>a8ae024</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1538,20 +1635,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>71</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -1559,7 +1656,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>72</v>
       </c>
@@ -1567,7 +1664,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>73</v>
       </c>
@@ -1575,7 +1672,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="314.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="314.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>75</v>
       </c>
@@ -1583,7 +1680,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>77</v>
       </c>
@@ -1591,7 +1688,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="233.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="233.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>79</v>
       </c>
@@ -1599,7 +1696,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>81</v>
       </c>
@@ -1607,7 +1704,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>83</v>
       </c>
@@ -1615,14 +1712,14 @@
         <v>46318</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>71</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="200" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="211.2" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>84</v>
       </c>
@@ -1630,7 +1727,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>85</v>
       </c>
@@ -1638,7 +1735,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>86</v>
       </c>
@@ -1646,7 +1743,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>87</v>
       </c>
@@ -1654,7 +1751,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>88</v>
       </c>
@@ -1662,11 +1759,69 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="3"/>
+      <c r="B17" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="211.2" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B21" s="18" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B22" s="19" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B23" s="19" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B24" s="20">
+        <v>46321</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B25" s="19" t="inlineStr">
+        <is>
+          <t>a8ae024</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1678,20 +1833,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>71</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -1699,7 +1854,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>72</v>
       </c>
@@ -1707,7 +1862,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>73</v>
       </c>
@@ -1715,7 +1870,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>75</v>
       </c>
@@ -1723,7 +1878,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>77</v>
       </c>
@@ -1731,7 +1886,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>79</v>
       </c>
@@ -1739,7 +1894,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>81</v>
       </c>
@@ -1747,7 +1902,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>83</v>
       </c>
@@ -1755,14 +1910,14 @@
         <v>46318</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>71</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="79.2" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>84</v>
       </c>
@@ -1770,7 +1925,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>85</v>
       </c>
@@ -1778,7 +1933,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>86</v>
       </c>
@@ -1786,7 +1941,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>87</v>
       </c>
@@ -1794,7 +1949,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>88</v>
       </c>
@@ -1802,14 +1957,73 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="3"/>
+      <c r="B17" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="79.2" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B23" s="17" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B24" s="12">
+        <v>46321</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>a8ae024</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1818,20 +2032,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>71</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -1839,7 +2053,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>72</v>
       </c>
@@ -1847,7 +2061,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>73</v>
       </c>
@@ -1855,7 +2069,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>75</v>
       </c>
@@ -1863,7 +2077,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>77</v>
       </c>
@@ -1871,7 +2085,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>79</v>
       </c>
@@ -1879,7 +2093,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>81</v>
       </c>
@@ -1887,7 +2101,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>83</v>
       </c>
@@ -1895,14 +2109,14 @@
         <v>46318</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>71</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="79.2" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>84</v>
       </c>
@@ -1910,7 +2124,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>85</v>
       </c>
@@ -1918,7 +2132,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>86</v>
       </c>
@@ -1926,7 +2140,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>87</v>
       </c>
@@ -1934,7 +2148,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>88</v>
       </c>
@@ -1942,11 +2156,69 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="3"/>
+      <c r="B17" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="79.2" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B23" s="17" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B24" s="12">
+        <v>46321</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>a8ae024</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1958,20 +2230,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>71</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -1979,7 +2251,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>72</v>
       </c>
@@ -1987,7 +2259,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>73</v>
       </c>
@@ -1995,7 +2267,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>75</v>
       </c>
@@ -2003,7 +2275,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>77</v>
       </c>
@@ -2011,7 +2283,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>79</v>
       </c>
@@ -2019,7 +2291,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>81</v>
       </c>
@@ -2027,7 +2299,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>83</v>
       </c>
@@ -2035,14 +2307,14 @@
         <v>46318</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>71</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="79.2" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>84</v>
       </c>
@@ -2050,7 +2322,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>85</v>
       </c>
@@ -2058,7 +2330,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>86</v>
       </c>
@@ -2066,7 +2338,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>87</v>
       </c>
@@ -2074,7 +2346,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>88</v>
       </c>
@@ -2082,11 +2354,69 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="3"/>
+      <c r="B17" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="79.2" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B21" s="18" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B22" s="19" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B23" s="19" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B24" s="20">
+        <v>46321</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B25" s="19" t="inlineStr">
+        <is>
+          <t>a8ae024</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2098,20 +2428,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>71</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -2119,7 +2449,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>72</v>
       </c>
@@ -2127,7 +2457,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>73</v>
       </c>
@@ -2135,7 +2465,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>75</v>
       </c>
@@ -2143,7 +2473,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>77</v>
       </c>
@@ -2151,7 +2481,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="112" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="112.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>79</v>
       </c>
@@ -2159,7 +2489,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>81</v>
       </c>
@@ -2167,7 +2497,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>83</v>
       </c>
@@ -2175,14 +2505,14 @@
         <v>46318</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>71</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="100" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="105.6" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>84</v>
       </c>
@@ -2190,7 +2520,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>85</v>
       </c>
@@ -2198,7 +2528,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>86</v>
       </c>
@@ -2206,7 +2536,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>87</v>
       </c>
@@ -2214,7 +2544,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>88</v>
       </c>
@@ -2222,11 +2552,69 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="3"/>
+      <c r="B17" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="105.6" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B21" s="18" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B22" s="19" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B23" s="19" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B24" s="20">
+        <v>46321</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B25" s="19" t="inlineStr">
+        <is>
+          <t>a8ae024</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2238,20 +2626,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>71</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -2259,7 +2647,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>72</v>
       </c>
@@ -2267,7 +2655,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>73</v>
       </c>
@@ -2275,7 +2663,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>75</v>
       </c>
@@ -2283,7 +2671,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>77</v>
       </c>
@@ -2291,7 +2679,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="112" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="112.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>79</v>
       </c>
@@ -2299,7 +2687,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>81</v>
       </c>
@@ -2307,7 +2695,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>83</v>
       </c>
@@ -2315,14 +2703,14 @@
         <v>46318</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>71</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="100" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="105.6" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>84</v>
       </c>
@@ -2330,7 +2718,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>85</v>
       </c>
@@ -2338,7 +2726,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>86</v>
       </c>
@@ -2346,7 +2734,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>87</v>
       </c>
@@ -2354,7 +2742,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>88</v>
       </c>
@@ -2362,11 +2750,69 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="3"/>
+      <c r="B17" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="105.6" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B21" s="18" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B22" s="19" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B23" s="19" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B24" s="20">
+        <v>46321</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B25" s="19" t="inlineStr">
+        <is>
+          <t>a8ae024</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2378,20 +2824,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>71</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -2399,7 +2845,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>72</v>
       </c>
@@ -2407,7 +2853,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>73</v>
       </c>
@@ -2415,7 +2861,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="382" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="382.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>75</v>
       </c>
@@ -2423,7 +2869,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="152.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="152.55000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>77</v>
       </c>
@@ -2439,7 +2885,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>81</v>
       </c>
@@ -2447,7 +2893,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>83</v>
       </c>
@@ -2455,14 +2901,14 @@
         <v>46318</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>71</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="400" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="409.6" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>84</v>
       </c>
@@ -2470,7 +2916,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>85</v>
       </c>
@@ -2478,7 +2924,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>86</v>
       </c>
@@ -2486,7 +2932,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>87</v>
       </c>
@@ -2494,7 +2940,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>88</v>
       </c>
@@ -2502,11 +2948,69 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="3"/>
+      <c r="B17" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="409.6" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B21" s="18" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B22" s="19" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B23" s="19" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B24" s="20">
+        <v>46321</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B25" s="19" t="inlineStr">
+        <is>
+          <t>a8ae024</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2518,20 +3022,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>71</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -2539,7 +3043,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>72</v>
       </c>
@@ -2547,7 +3051,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>73</v>
       </c>
@@ -2555,7 +3059,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="395.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="395.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>75</v>
       </c>
@@ -2563,7 +3067,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="152.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="152.55000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>77</v>
       </c>
@@ -2579,7 +3083,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>81</v>
       </c>
@@ -2587,7 +3091,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>83</v>
       </c>
@@ -2595,14 +3099,14 @@
         <v>46318</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>71</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="409.6" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>84</v>
       </c>
@@ -2610,7 +3114,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>85</v>
       </c>
@@ -2618,7 +3122,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>86</v>
       </c>
@@ -2626,7 +3130,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>87</v>
       </c>
@@ -2634,7 +3138,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>88</v>
       </c>
@@ -2642,11 +3146,69 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="3"/>
+      <c r="B17" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="409.6" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B21" s="18" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B22" s="19" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B23" s="19" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B24" s="20">
+        <v>46321</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B25" s="19" t="inlineStr">
+        <is>
+          <t>a8ae024</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2658,20 +3220,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>71</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -2679,7 +3241,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>72</v>
       </c>
@@ -2687,7 +3249,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>73</v>
       </c>
@@ -2703,7 +3265,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="152.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="152.55000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>77</v>
       </c>
@@ -2719,7 +3281,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>81</v>
       </c>
@@ -2727,7 +3289,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>83</v>
       </c>
@@ -2735,14 +3297,14 @@
         <v>46318</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>71</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="409.6" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>84</v>
       </c>
@@ -2750,7 +3312,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>85</v>
       </c>
@@ -2758,7 +3320,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>86</v>
       </c>
@@ -2766,7 +3328,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>87</v>
       </c>
@@ -2774,7 +3336,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>88</v>
       </c>
@@ -2782,11 +3344,69 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="3"/>
+      <c r="B17" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="409.6" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B21" s="18" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B22" s="19" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B23" s="19" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B24" s="20">
+        <v>46321</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B25" s="19" t="inlineStr">
+        <is>
+          <t>a8ae024</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
SPM-94: Record the TC11 manual run (pass)
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-94_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-94_Test_Cases.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\IS212\docs\test-cases\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\krist\Documents\GitHub\IS212\docs\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9C4E33B-8A04-4EAE-8448-0A12BF2291E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA0D1A6D-B135-42A0-BDDB-25AE4FBD02DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" firstSheet="9" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14730" yWindow="-16200" windowWidth="14610" windowHeight="15585" firstSheet="9" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="551" uniqueCount="131">
   <si>
     <t>Item</t>
   </si>
@@ -600,6 +600,9 @@
 Step 7: The All events list shows SPM94 Meridian Cancelled Approved Expo with the status 'Cancelled'. SPM94 Meridian Cancelled Review Dinner is not listed.
 Step 8: The event page opens with the title SPM94 Meridian Cancelled Approved Expo and the status 'Cancelled'.
 Step 9: SPM94 Meridian Cancelled Review Dinner was never approved, so the page heading reads 'Event' and an error box titled 'Could not load this' says 'This event doesn't exist, or you don't have access to it.', with a 'Retry' button. No event title, status or rejection reason is shown.</t>
+  </si>
+  <si>
+    <t>f67205a</t>
   </si>
 </sst>
 </file>
@@ -795,12 +798,12 @@
     <xf numFmtId="164" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -818,55 +821,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>679666</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>1809843</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{13DBF453-980F-6D0B-F5FC-83C7AC747538}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5702300" y="1174750"/>
-          <a:ext cx="4210266" cy="1809843"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1068,7 +1022,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I23"/>
-  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -1081,11 +1035,11 @@
     <col min="9" max="9" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="17" t="s">
         <v>29</v>
       </c>
       <c r="C1" s="18"/>
@@ -1096,7 +1050,7 @@
       <c r="H1" s="18"/>
       <c r="I1" s="19"/>
     </row>
-    <row r="3" spans="1:9" ht="13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>30</v>
       </c>
@@ -1275,7 +1229,7 @@
       <c r="H9" s="9"/>
       <c r="I9" s="9"/>
     </row>
-    <row r="10" spans="1:9" ht="39.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>64</v>
       </c>
@@ -1300,7 +1254,7 @@
       <c r="H10" s="9"/>
       <c r="I10" s="9"/>
     </row>
-    <row r="11" spans="1:9" ht="39.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>67</v>
       </c>
@@ -1375,7 +1329,7 @@
       <c r="H13" s="9"/>
       <c r="I13" s="9"/>
     </row>
-    <row r="14" spans="1:9" ht="25" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
         <v>77</v>
       </c>
@@ -1400,136 +1354,136 @@
       <c r="H14" s="9"/>
       <c r="I14" s="9"/>
     </row>
-    <row r="16" spans="1:9" ht="13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="B16" s="20" t="s">
+      <c r="B16" s="17" t="s">
         <v>82</v>
       </c>
       <c r="C16" s="18"/>
       <c r="D16" s="19"/>
-      <c r="E16" s="20" t="s">
+      <c r="E16" s="17" t="s">
         <v>83</v>
       </c>
       <c r="F16" s="19"/>
     </row>
-    <row r="17" spans="1:6" ht="71.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" ht="71.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="20" t="s">
         <v>84</v>
       </c>
       <c r="C17" s="18"/>
       <c r="D17" s="19"/>
-      <c r="E17" s="17" t="s">
+      <c r="E17" s="20" t="s">
         <v>85</v>
       </c>
       <c r="F17" s="19"/>
     </row>
-    <row r="18" spans="1:6" ht="85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="20" t="s">
         <v>86</v>
       </c>
       <c r="C18" s="18"/>
       <c r="D18" s="19"/>
-      <c r="E18" s="17" t="s">
+      <c r="E18" s="20" t="s">
         <v>87</v>
       </c>
       <c r="F18" s="19"/>
     </row>
-    <row r="19" spans="1:6" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="B19" s="17" t="s">
+      <c r="B19" s="20" t="s">
         <v>89</v>
       </c>
       <c r="C19" s="18"/>
       <c r="D19" s="19"/>
-      <c r="E19" s="17" t="s">
+      <c r="E19" s="20" t="s">
         <v>52</v>
       </c>
       <c r="F19" s="19"/>
     </row>
-    <row r="20" spans="1:6" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="B20" s="20" t="s">
         <v>91</v>
       </c>
       <c r="C20" s="18"/>
       <c r="D20" s="19"/>
-      <c r="E20" s="17" t="s">
+      <c r="E20" s="20" t="s">
         <v>57</v>
       </c>
       <c r="F20" s="19"/>
     </row>
-    <row r="21" spans="1:6" ht="71.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" ht="71.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="20" t="s">
         <v>93</v>
       </c>
       <c r="C21" s="18"/>
       <c r="D21" s="19"/>
-      <c r="E21" s="17" t="s">
+      <c r="E21" s="20" t="s">
         <v>94</v>
       </c>
       <c r="F21" s="19"/>
     </row>
-    <row r="22" spans="1:6" ht="71.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" ht="71.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="B22" s="17" t="s">
+      <c r="B22" s="20" t="s">
         <v>96</v>
       </c>
       <c r="C22" s="18"/>
       <c r="D22" s="19"/>
-      <c r="E22" s="17" t="s">
+      <c r="E22" s="20" t="s">
         <v>97</v>
       </c>
       <c r="F22" s="19"/>
     </row>
-    <row r="23" spans="1:6" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="B23" s="17" t="s">
+      <c r="B23" s="20" t="s">
         <v>99</v>
       </c>
       <c r="C23" s="18"/>
       <c r="D23" s="19"/>
-      <c r="E23" s="17" t="s">
+      <c r="E23" s="20" t="s">
         <v>71</v>
       </c>
       <c r="F23" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="B21:D21"/>
     <mergeCell ref="B1:I1"/>
     <mergeCell ref="B16:D16"/>
     <mergeCell ref="B20:D20"/>
     <mergeCell ref="B19:D19"/>
     <mergeCell ref="E20:F20"/>
     <mergeCell ref="E16:F16"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="E19:F19"/>
     <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="B21:D21"/>
     <mergeCell ref="E17:F17"/>
   </mergeCells>
   <hyperlinks>
@@ -1555,19 +1509,19 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:C25"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -1575,7 +1529,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -1583,7 +1537,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -1591,7 +1545,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="152.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="152.55000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
@@ -1599,7 +1553,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
@@ -1607,7 +1561,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="179.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="179.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
@@ -1615,7 +1569,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
@@ -1623,7 +1577,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>15</v>
       </c>
@@ -1631,14 +1585,14 @@
         <v>46318</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="171.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="171.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>16</v>
       </c>
@@ -1646,7 +1600,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -1654,7 +1608,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>19</v>
       </c>
@@ -1662,7 +1616,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>21</v>
       </c>
@@ -1670,7 +1624,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>23</v>
       </c>
@@ -1678,7 +1632,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>24</v>
       </c>
@@ -1686,13 +1640,13 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B19" s="5"/>
     </row>
-    <row r="20" spans="1:2" ht="171.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" ht="171.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>16</v>
       </c>
@@ -1751,19 +1705,19 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:C25"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -1771,7 +1725,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -1779,7 +1733,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -1787,7 +1741,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="314.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="314.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
@@ -1795,7 +1749,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
@@ -1803,7 +1757,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="233.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="233.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
@@ -1811,7 +1765,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
@@ -1819,7 +1773,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>15</v>
       </c>
@@ -1827,14 +1781,14 @@
         <v>46318</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="211.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="211.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>16</v>
       </c>
@@ -1842,7 +1796,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -1850,7 +1804,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>19</v>
       </c>
@@ -1858,7 +1812,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>21</v>
       </c>
@@ -1866,7 +1820,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>23</v>
       </c>
@@ -1874,7 +1828,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>24</v>
       </c>
@@ -1882,13 +1836,13 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B19" s="5"/>
     </row>
-    <row r="20" spans="1:2" ht="211.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" ht="211.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>16</v>
       </c>
@@ -1946,20 +1900,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -1967,7 +1921,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -1975,7 +1929,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -1983,7 +1937,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="193" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="193.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
@@ -1991,7 +1945,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="112" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="112.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
@@ -1999,7 +1953,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="179.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="179.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
@@ -2007,7 +1961,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
@@ -2015,7 +1969,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>15</v>
       </c>
@@ -2023,14 +1977,14 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="162.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="171.6" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>16</v>
       </c>
@@ -2038,7 +1992,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -2046,7 +2000,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>19</v>
       </c>
@@ -2054,7 +2008,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>21</v>
       </c>
@@ -2062,7 +2016,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>23</v>
       </c>
@@ -2070,20 +2024,72 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="3" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="211.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" s="15" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24" s="16">
+        <v>46321</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25" s="15" t="inlineStr">
         <is>
-          <t>f67205a</t>
+          <t>5c3fc31</t>
         </is>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="211.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2093,19 +2099,19 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:C25"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -2113,7 +2119,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -2121,7 +2127,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -2129,7 +2135,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
@@ -2137,7 +2143,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
@@ -2145,7 +2151,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
@@ -2153,7 +2159,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
@@ -2161,7 +2167,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>15</v>
       </c>
@@ -2169,14 +2175,14 @@
         <v>46318</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="79.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="79.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>16</v>
       </c>
@@ -2184,7 +2190,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -2192,7 +2198,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>19</v>
       </c>
@@ -2200,7 +2206,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>21</v>
       </c>
@@ -2208,7 +2214,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>23</v>
       </c>
@@ -2216,7 +2222,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>24</v>
       </c>
@@ -2224,13 +2230,13 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B19" s="5"/>
     </row>
-    <row r="20" spans="1:2" ht="79.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" ht="79.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>16</v>
       </c>
@@ -2290,19 +2296,19 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:C25"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -2310,7 +2316,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -2318,7 +2324,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -2326,7 +2332,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
@@ -2334,7 +2340,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
@@ -2342,7 +2348,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
@@ -2350,7 +2356,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
@@ -2358,7 +2364,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>15</v>
       </c>
@@ -2366,14 +2372,14 @@
         <v>46318</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="79.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="79.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>16</v>
       </c>
@@ -2381,7 +2387,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -2389,7 +2395,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>19</v>
       </c>
@@ -2397,7 +2403,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>21</v>
       </c>
@@ -2405,7 +2411,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>23</v>
       </c>
@@ -2413,7 +2419,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>24</v>
       </c>
@@ -2421,13 +2427,13 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B19" s="5"/>
     </row>
-    <row r="20" spans="1:2" ht="79.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" ht="79.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>16</v>
       </c>
@@ -2486,19 +2492,19 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:C25"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -2506,7 +2512,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -2514,7 +2520,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -2522,7 +2528,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
@@ -2530,7 +2536,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
@@ -2538,7 +2544,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
@@ -2546,7 +2552,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
@@ -2554,7 +2560,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>15</v>
       </c>
@@ -2562,14 +2568,14 @@
         <v>46318</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="79.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="79.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>16</v>
       </c>
@@ -2577,7 +2583,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -2585,7 +2591,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>19</v>
       </c>
@@ -2593,7 +2599,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>21</v>
       </c>
@@ -2601,7 +2607,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>23</v>
       </c>
@@ -2609,7 +2615,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>24</v>
       </c>
@@ -2617,13 +2623,13 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B19" s="5"/>
     </row>
-    <row r="20" spans="1:2" ht="79.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" ht="79.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>16</v>
       </c>
@@ -2682,19 +2688,19 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:C25"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -2702,7 +2708,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -2710,7 +2716,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -2718,7 +2724,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
@@ -2726,7 +2732,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
@@ -2734,7 +2740,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="112" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="112.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
@@ -2742,7 +2748,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
@@ -2750,7 +2756,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>15</v>
       </c>
@@ -2758,14 +2764,14 @@
         <v>46318</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="105.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="105.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>16</v>
       </c>
@@ -2773,7 +2779,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -2781,7 +2787,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>19</v>
       </c>
@@ -2789,7 +2795,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>21</v>
       </c>
@@ -2797,7 +2803,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>23</v>
       </c>
@@ -2805,7 +2811,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>24</v>
       </c>
@@ -2813,13 +2819,13 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B19" s="5"/>
     </row>
-    <row r="20" spans="1:2" ht="105.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" ht="105.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>16</v>
       </c>
@@ -2878,19 +2884,19 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:C25"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -2898,7 +2904,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -2906,7 +2912,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -2914,7 +2920,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
@@ -2922,7 +2928,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
@@ -2930,7 +2936,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="112" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="112.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
@@ -2938,7 +2944,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
@@ -2946,7 +2952,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>15</v>
       </c>
@@ -2954,14 +2960,14 @@
         <v>46318</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="105.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="105.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>16</v>
       </c>
@@ -2969,7 +2975,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -2977,7 +2983,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>19</v>
       </c>
@@ -2985,7 +2991,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>21</v>
       </c>
@@ -2993,7 +2999,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>23</v>
       </c>
@@ -3001,7 +3007,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>24</v>
       </c>
@@ -3009,13 +3015,13 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B19" s="5"/>
     </row>
-    <row r="20" spans="1:2" ht="105.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" ht="105.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>16</v>
       </c>
@@ -3074,19 +3080,19 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:C25"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -3094,7 +3100,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -3102,7 +3108,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -3110,7 +3116,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="382" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="382.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
@@ -3118,7 +3124,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="152.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="152.55000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
@@ -3134,7 +3140,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
@@ -3142,7 +3148,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>15</v>
       </c>
@@ -3150,7 +3156,7 @@
         <v>46318</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
@@ -3165,7 +3171,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -3173,7 +3179,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>19</v>
       </c>
@@ -3181,7 +3187,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>21</v>
       </c>
@@ -3189,7 +3195,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>23</v>
       </c>
@@ -3197,7 +3203,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>24</v>
       </c>
@@ -3205,7 +3211,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>0</v>
       </c>
@@ -3270,19 +3276,19 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:C25"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -3290,7 +3296,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -3298,7 +3304,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -3306,7 +3312,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="395.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="395.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
@@ -3314,7 +3320,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="152.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="152.55000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
@@ -3330,7 +3336,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
@@ -3338,7 +3344,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>15</v>
       </c>
@@ -3346,7 +3352,7 @@
         <v>46318</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
@@ -3361,7 +3367,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -3369,7 +3375,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>19</v>
       </c>
@@ -3377,7 +3383,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>21</v>
       </c>
@@ -3385,7 +3391,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>23</v>
       </c>
@@ -3393,7 +3399,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>24</v>
       </c>
@@ -3401,7 +3407,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>0</v>
       </c>
@@ -3466,19 +3472,19 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:C25"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -3486,7 +3492,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -3494,7 +3500,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -3510,7 +3516,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="152.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="152.55000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
@@ -3526,7 +3532,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
@@ -3534,7 +3540,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>15</v>
       </c>
@@ -3542,7 +3548,7 @@
         <v>46318</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
@@ -3557,7 +3563,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -3565,7 +3571,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>19</v>
       </c>
@@ -3573,7 +3579,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>21</v>
       </c>
@@ -3581,7 +3587,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>23</v>
       </c>
@@ -3589,7 +3595,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>24</v>
       </c>
@@ -3597,7 +3603,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>0</v>
       </c>

</xml_diff>